<commit_message>
Import flux Century 21, type Triplex et badge Localisation exacte
- Type de bien Triplex (enum, migration, formulaire, filtres, fiches), champs identiques au duplex
- Annonces : colonnes source/source_id/source_url ; badge "Localisation exacte" sur les annonces publiées sur Localizi
- backend/import_century21.py : import/synchronisation du flux XML (12 comptes agence, statut en_attente, prix 0 -> 1 DT, décalage des points, retrait des annonces disparues)
- Référentiel : "Berge du Lac" -> "Berges du Lac" (migration + xlsx), Jardins de Carthage sous El Kram
- Ajout du rapport de conception

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/data/tunisie.xlsx
+++ b/backend/data/tunisie.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4870"/>
+  <dimension ref="A1:C4871"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -79185,7 +79185,7 @@
       </c>
       <c r="C4633" t="inlineStr">
         <is>
-          <t>BERGE DU LAC</t>
+          <t>BERGES DU LAC</t>
         </is>
       </c>
     </row>
@@ -83215,6 +83215,23 @@
       <c r="C4870" t="inlineStr">
         <is>
           <t>ZEGUIDANE</t>
+        </is>
+      </c>
+    </row>
+    <row r="4871">
+      <c r="A4871" t="inlineStr">
+        <is>
+          <t>TUNIS</t>
+        </is>
+      </c>
+      <c r="B4871" t="inlineStr">
+        <is>
+          <t>EL KRAM</t>
+        </is>
+      </c>
+      <c r="C4871" t="inlineStr">
+        <is>
+          <t>JARDINS DE CARTHAGE</t>
         </is>
       </c>
     </row>

</xml_diff>